<commit_message>
Refactor: Alteração na geração do Excel consilidando de forma unica a gravaçao
</commit_message>
<xml_diff>
--- a/Resultado_Busca.xlsx
+++ b/Resultado_Busca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,36 +443,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CSC00900</t>
+          <t>CS00000M</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CS00000F, CS00000M, CS00000S, CS00001M</t>
+          <t>CS00000S</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CSC00903</t>
+          <t>CSC00900</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CS00000M, CS00000S, CS00001M</t>
+          <t>CS00000F, CS00000M, CS00000S, CS00001M</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CSF00000</t>
+          <t>CSC00903</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nenhuma referencia encontrada</t>
+          <t>CS00000M, CS00000S, CS00001M</t>
         </is>
       </c>
     </row>
@@ -485,42 +485,6 @@
       <c r="B5" t="inlineStr">
         <is>
           <t>CS00000M, CS00001M</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CSF00200</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Nenhuma referencia encontrada</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CSF00300</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Nenhuma referencia encontrada</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CSF33300</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Nenhuma referencia encontrada</t>
         </is>
       </c>
     </row>

</xml_diff>